<commit_message>
bpom_audit_stock: update SKU/BPOM master (66 rows)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bpom_audit_stock/reference/Data SKU BPOM.xlsx
+++ b/bpom_audit_stock/reference/Data SKU BPOM.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yulian Farid\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07408E8C-C780-45BC-8658-F3F1EF44024E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B25A97E2-390A-4EEC-A0CA-4CB0BE643D03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{01CE1EA7-1E13-484C-AEA9-BF021F85F2D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$72</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="87">
   <si>
     <t>SKU</t>
   </si>
@@ -137,9 +140,6 @@
     <t>NA11251700100</t>
   </si>
   <si>
-    <t>SKINTIFIC-28</t>
-  </si>
-  <si>
     <t>SKINTIFIC-30</t>
   </si>
   <si>
@@ -240,9 +240,6 @@
   </si>
   <si>
     <t>SKINTIFIC-122</t>
-  </si>
-  <si>
-    <t>SKINTIFIC-172</t>
   </si>
   <si>
     <t>SKINTIFIC-09</t>
@@ -802,7 +799,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -894,13 +891,13 @@
     </row>
     <row r="8" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D8" s="8">
         <v>46369</v>
@@ -908,13 +905,13 @@
     </row>
     <row r="9" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B9" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>71</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>73</v>
       </c>
       <c r="D9" s="8">
         <v>46620</v>
@@ -922,13 +919,13 @@
     </row>
     <row r="10" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D10" s="8">
         <v>46634</v>
@@ -936,13 +933,13 @@
     </row>
     <row r="11" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D11" s="8">
         <v>47010</v>
@@ -1006,13 +1003,13 @@
     </row>
     <row r="16" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D16" s="8">
         <v>46388</v>
@@ -1020,13 +1017,13 @@
     </row>
     <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B17" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>76</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>78</v>
       </c>
       <c r="D17" s="8">
         <v>47024</v>
@@ -1090,128 +1087,128 @@
     </row>
     <row r="22" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D22" s="8">
-        <v>46388</v>
+        <v>47026</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D23" s="8">
-        <v>47024</v>
+        <v>46990</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>80</v>
       </c>
       <c r="D24" s="8">
-        <v>47026</v>
+        <v>46382</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>81</v>
       </c>
       <c r="D25" s="8">
-        <v>46990</v>
+        <v>46636</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D26" s="8">
-        <v>46382</v>
+        <v>47013</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D27" s="8">
-        <v>46636</v>
+        <v>47069</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>85</v>
       </c>
       <c r="D28" s="8">
-        <v>47013</v>
+        <v>47150</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="7" t="s">
-        <v>70</v>
+        <v>26</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>84</v>
+        <v>27</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>86</v>
+        <v>28</v>
       </c>
       <c r="D29" s="8">
-        <v>47069</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="7" t="s">
-        <v>70</v>
+        <v>26</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>84</v>
+        <v>27</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>87</v>
+        <v>29</v>
       </c>
       <c r="D30" s="8">
-        <v>47150</v>
+        <v>46870</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1222,10 +1219,10 @@
         <v>27</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D31" s="8">
-        <v>46282</v>
+        <v>47243</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1236,38 +1233,38 @@
         <v>27</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D32" s="8">
-        <v>46870</v>
+        <v>46943</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="7" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="D33" s="8">
-        <v>47243</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="7" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="D34" s="8">
-        <v>46943</v>
+        <v>47322</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1278,80 +1275,80 @@
         <v>4</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D35" s="8">
-        <v>46179</v>
+        <v>46990</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="7" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="D36" s="8">
-        <v>47322</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="7" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="D37" s="8">
-        <v>46990</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="7" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="D38" s="8">
-        <v>46179</v>
+        <v>46481</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="7" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="D39" s="8">
-        <v>47322</v>
+        <v>47236</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="7" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="D40" s="8">
-        <v>46990</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1359,13 +1356,13 @@
         <v>40</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D41" s="8">
-        <v>46282</v>
+        <v>47017</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1373,139 +1370,139 @@
         <v>40</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="D42" s="8">
-        <v>46255</v>
+        <v>47320</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="7" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="D43" s="8">
-        <v>46481</v>
+        <v>47133</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A44" s="7" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D44" s="8">
-        <v>47236</v>
+        <v>45970</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="D45" s="8">
-        <v>46167</v>
+        <v>46383</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D46" s="8">
-        <v>47017</v>
+        <v>47139</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="7" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="D47" s="8">
-        <v>47320</v>
+        <v>47006</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="7" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="D48" s="8">
-        <v>47133</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="7" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D49" s="8">
-        <v>45970</v>
+        <v>46969</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A50" s="7" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="D50" s="8">
-        <v>46383</v>
+        <v>45981</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="7" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="D51" s="8">
-        <v>47139</v>
+        <v>46494</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1513,83 +1510,83 @@
         <v>57</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="D52" s="8">
-        <v>47006</v>
+        <v>47294</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="7" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="D53" s="8">
-        <v>46313</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="7" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="D54" s="8">
-        <v>46969</v>
+        <v>46870</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="7" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="D55" s="8">
-        <v>45981</v>
+        <v>47243</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="7" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="D56" s="8">
-        <v>46494</v>
+        <v>46943</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A57" s="7" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="D57" s="8">
-        <v>47294</v>
+        <v>46026</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1597,13 +1594,13 @@
         <v>63</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D58" s="8">
-        <v>46282</v>
+        <v>46481</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1611,13 +1608,13 @@
         <v>63</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D59" s="8">
-        <v>46870</v>
+        <v>46614</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1625,69 +1622,69 @@
         <v>63</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D60" s="8">
-        <v>47243</v>
+        <v>47010</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="7" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>31</v>
+        <v>78</v>
       </c>
       <c r="D61" s="8">
-        <v>46943</v>
+        <v>47026</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="7" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>21</v>
+        <v>79</v>
       </c>
       <c r="D62" s="8">
-        <v>46026</v>
+        <v>46990</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A63" s="7" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>22</v>
+        <v>77</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>23</v>
+        <v>80</v>
       </c>
       <c r="D63" s="8">
-        <v>46481</v>
+        <v>46382</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="7" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>22</v>
+        <v>77</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="D64" s="8">
-        <v>46614</v>
+        <v>46636</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1695,112 +1692,72 @@
         <v>64</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="D65" s="8">
-        <v>47010</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="7" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="D66" s="8">
-        <v>47026</v>
+        <v>47017</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A67" s="7" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
       <c r="D67" s="8">
-        <v>46990</v>
+        <v>47320</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A68" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="B68" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="C68" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="D68" s="8">
-        <v>46382</v>
-      </c>
+      <c r="A68" s="7"/>
+      <c r="B68" s="7"/>
+      <c r="C68" s="7"/>
+      <c r="D68" s="8"/>
     </row>
     <row r="69" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A69" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="B69" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="C69" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="D69" s="8">
-        <v>46636</v>
-      </c>
+      <c r="A69" s="7"/>
+      <c r="B69" s="7"/>
+      <c r="C69" s="7"/>
+      <c r="D69" s="8"/>
     </row>
     <row r="70" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A70" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B70" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C70" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D70" s="8">
-        <v>46167</v>
-      </c>
+      <c r="A70" s="7"/>
+      <c r="B70" s="7"/>
+      <c r="C70" s="7"/>
+      <c r="D70" s="8"/>
     </row>
     <row r="71" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A71" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B71" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C71" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D71" s="8">
-        <v>47017</v>
-      </c>
+      <c r="A71" s="7"/>
+      <c r="B71" s="7"/>
+      <c r="C71" s="7"/>
+      <c r="D71" s="8"/>
     </row>
     <row r="72" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A72" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B72" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C72" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="D72" s="8">
-        <v>47320</v>
-      </c>
+      <c r="A72" s="7"/>
+      <c r="B72" s="7"/>
+      <c r="C72" s="7"/>
+      <c r="D72" s="8"/>
     </row>
     <row r="73" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="3"/>
@@ -1875,6 +1832,7 @@
       <c r="D84" s="4"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D72" xr:uid="{0D48195E-081D-4623-A4A5-F9DBA399A697}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>